<commit_message>
fix: strip Japanese kana + Korean hangul from patent data, fix GBK crash in compile_pdf
- Patent applicant/inventor fields may contain JP/KR characters that break xelatex
- Clean via Unicode range removal (Hiragana+Katakana+Hangul)
- Also fix print(out[-2000:]) GBK crash on LaTeX error output

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/weekly_temp/patents_低温环境系统.xlsx
+++ b/weekly_temp/patents_低温环境系统.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,222 +456,74 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>用于在低温工作温度下操作一组量子比特的系统和方法</t>
+          <t>接收方小型化量子密钥生成终端</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>荷兰应用自然科学研究组织</t>
+          <t>科大国盾量子技术股份有限公司</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VAN ZWET, ERWIN JOHN</t>
+          <t>杜先常 | 唐世彪 | 陈国靖 | 董军</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>公开专利</t>
+          <t>授权专利</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>本发明提供了一种用于在低温工作温度 (Tq) 下操作一组量子位 (10q) 的系统 (100) 和方法。该系统包括第一基板 (10) 和第二基板 (20),它们通过一组连接器 (30) 电连接。第一基板 (10) 包含一组量子位 (10q),第二基板 (20) 包含配置用于操作该组量子位 (10q) 的电子器件 (21)。第一冷却元件 (41) 将第一基板 (10) 保持在低于低温工作温度 (Tq) 的第一低温温度 (T1),第二冷却元件 (42) 将第二基板 (20) 保持在高于低温工作温度 (Tq) 的第二低温温度 (T2)。该组连接器(30)被配置为将第二基板(20)和第一基板(10)之间的热流保持在足够低的阈值以下,以将一组量子位(10q)维持在低温工作温度(Tq)。</t>
+          <t>本发明提供一种接收方小型化量子密钥生成终端，包括机箱(1)、主控板(2)、探测器模块(3)、解码光路(4)、电源(5)和风扇(6)，主控板(2)和解码光路(4)左右并排设置，并且主控板(2)和解码光路(4)的前端抵在机箱(1)的前面板的内部，探测器模块(3)与解码光路(4)前后并排设置，且探测器模块(3)与解码光路(4)的左端部均紧挨主控板(2)的右端部；电源(5)设置在机箱(1)的后部，吹风风扇(6)设置在靠近探测器模块(3)的一侧。本发明的优点在于：在保证通信可靠性的前提下实现了接收方量子密钥生成终端的小型化，经热仿真和力仿真测试，热设计和力设计满足设备使用要求。</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=8f619a02-cea9-462f-9e6e-4dca613a46ae&amp;shareId=E41F3B0F-9352-71B8-3F94-09F7G7CDE08G&amp;from=EXPORT&amp;signature=AHBRRSlZDoMjNQwrWLsszX7nPvGbNQFEffsWap38SDI%3D&amp;expire=94608000&amp;date=20260529T004228Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=f4921438-27c2-41b2-a5af-afb2aa2b757f&amp;shareId=9822D43G-CCG6-9909-3EB1-2F5994384B2D&amp;from=EXPORT&amp;signature=IekkCgLKSsSp53YhWWg8X8KWGbrIraDcr9lDYUnXcIY%3D&amp;expire=94608000&amp;date=20260605T003852Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>一种基于热电转换效应的笔记本电脑废热回收利用系统及方法</t>
+          <t>采用量子处理单元(QPU)的图形处理单元(GPU)叠加计算系统</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>百信信息技术有限公司 | 安徽百信信息技术有限公司</t>
+          <t>芯科量子公司</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>王宪朝 | 鞠荣荣 | 汪玲 | 陶方强 | 黄巧林 | 曾盛坚 | 胡晓雨</t>
+          <t>ハッチングス, マシュー | ムカノフ, オレグ | レヴィ, ジョン</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>授权专利</t>
+          <t>公开专利</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>本发明公开了一种基于热电转换效应的笔记本电脑废热回收利用系统及方法，涉及热电材料与器件技术领域，包括：分布式热电阵列模块：由多个微型TEG单元组成，分布于笔记本高发热区域，通过温差直接发电；自适应热管理模块：包括导热硅胶层与微型散热鳍片，优化热端与冷端的温差；多级电能管理模块：包括整流电路、DC‑DC升压芯片及回收储能电池装置，将TEG输出的不稳定低压直流电转换为稳定电能，储存后供给目标设备；智能控制模块：根据温度传感器数据动态调整微型热电发电单元的工作区域，优先选择温差最大的位置发电，并通过PMIC芯片匹配供电需求。本发明通过创新设计实现废热高效转换及利用，解决小型化设备中热电转换效率低的问题，实现节能与环保。</t>
+          <t>本专利文件提供了一种高效的量子-经典混合计算系统的设计方案,该系统能够基于量子计算(利用量子比特的不同量子态)和经典数字计算(利用包含一个或多个图形处理单元(GPU)处理器的数字处理器)进行信息处理。本发明提供了一种采用量子处理单元(QPU)的图形处理单元(GPU)叠加计算系统。</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=79c9d744-08d0-473f-a097-08a12218cd8d&amp;shareId=E41F3B0F-9352-71B8-3F94-09F7G7CDE08G&amp;from=EXPORT&amp;signature=SQaExLyYD5Q3%2BfTRTRBNRh3wn8E6JLI36uURJgZpuYc%3D&amp;expire=94608000&amp;date=20260529T004228Z&amp;version=1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>温度梯度控制的蒸发造粒塔制备煤基量子碳点缓释肥料的方法</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>北京天中树科技发展有限公司</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>吴则昀 | 吴则一 | 朱光华</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>授权专利</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>本发明提供了温度梯度控制的蒸发造粒塔制备煤基量子碳点缓释肥料的方法，涉及农业肥料制备技术领域，包括在蒸发造粒塔内部自下至上设置高温区、中温区和低温区、煤粉与超临界水混合在高温区反应生成量子碳点前驱体、量子碳点前驱体在中温区内部通过氨气吹扫后与硼酸溶液反应、碳点溶液与尿素熔融液混合、双混液在低温区通过双流体喷嘴雾化形成复合肥料颗粒、在流化床包衣机内喷入氧化海藻酸钠/聚乙二醇复合膜溶液对复合肥料颗粒进行包衣；本发明在蒸发造粒塔内部自下至上设置高温区、中温区和低温区，实现将量子碳点合成、表面修饰、肥料复合三大核心工序集成于同一设备内，避免了跨设备操作导致的量子碳点结构破坏，保证产物稳定性。</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=2bee4aa4-7314-4d65-bd8f-580b34cdbd8a&amp;shareId=E41F3B0F-9352-71B8-3F94-09F7G7CDE08G&amp;from=EXPORT&amp;signature=u2YngjdHVkBZdvCJNaUqLtPNSreVyoIsxHyVwGhVzaY%3D&amp;expire=94608000&amp;date=20260529T004228Z&amp;version=1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>一种高浓度尿素废水中非挥发性酸根定向去除与尿素回收的方法和系统</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>宜兴鸿微环保科技有限公司</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>李侃 | 高启新 | 华佳 | 安丽娟</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>公开专利</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>本发明公开了一种高浓度尿素废水中非挥发性酸根定向去除与尿素回收的方法和系统，属于废水处理与资源回收技术领域。该方法先将废水引入预处理单元，投加碱金属盐、有机络合剂与纳米催化颗粒复配而成的协同处理剂，定向沉淀非挥发性酸根形成致密沉淀物；再通过超声辅助卧式螺旋卸料沉降离心机完成强化固液分离，上清液经石墨烯量子点‑温度响应性磁性纳米粒子复合改性阴离子交换树脂深度吸附残留酸根，实现酸根近乎完全去除；随后采用低温蒸发‑余热回收耦合工艺浓缩尿素，经分段温度‑压力梯度结晶析出高纯度尿素晶体；吸附饱和的树脂通过磁场分离回收，经温度调控温和再生后循环复用；适用于工业高浓度尿素废水资源化处理。</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=9d646539-046f-4512-a61b-935b36551599&amp;shareId=E41F3B0F-9352-71B8-3F94-09F7G7CDE08G&amp;from=EXPORT&amp;signature=jhY6zmTgOZsn%2BHBeS26e7YxBuQimizNLsLFV7Jpn604%3D&amp;expire=94608000&amp;date=20260529T004228Z&amp;version=1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>一种高性能深紫外发光器件及其制备方法</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>北京大学</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>王新强 | 李泰 | 刘放 | 马文结 | 袁泽兴 | 刘一欣 | 王超雨 | 王平</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>公开专利</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>本发明公开了一种高性能深紫外发光器件及其制备方法，属于半导体外延生长技术领域。本发明通过构建预制压应力结合受限减薄的协同机制，制备超薄量子阱并引入有效的压应力，以实现能带调控提升量子阱的TE偏振发光占比，解决了现有深紫外发光器件中量子阱应力引入与结构稳定性难以兼顾的技术难题。第二超晶格层使随后外延的量子阱在生长过程中受到受控的外部压应力；通过受控减薄形成的超薄量子阱具有增强的量子限制效应，与预置压应力协同作用，使价带顶态的能量排序向有利于TE跃迁的方向移动，从而有效抑制TM分量并显著提升TE发光占比。本发明为深紫外发光器件在紫外消毒、医疗、环境监测及精密光学等领域的应用提供了可行的制备基础。</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=26d84603-c7ad-444d-b34d-4e57623f1ad3&amp;shareId=E41F3B0F-9352-71B8-3F94-09F7G7CDE08G&amp;from=EXPORT&amp;signature=qYosjKe3ZQri2d4ISd9KCR0rTig2acL9jIeLeLwqaCw%3D&amp;expire=94608000&amp;date=20260529T004228Z&amp;version=1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>用于量子计算测控的集成滤波放大装置</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>相干(北京)科技有限公司</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>赵剑琴 | 邢磊 | 田建强 | 贺玉龙 | 曾祥洪</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>授权专利</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>本申请涉及一种用于量子计算测控的集成滤波放大装置，包括：装置壳体、电路板、前端衰减组件、前端带通滤波组件、微波放大组件、后端衰减组件和后端带通滤波组件，前端带通滤波组件、前端衰减组件、微波放大组件、后端衰减组件和后端带通滤波组件，依次连接设置在所述电路板上，且均集成在装置壳体内，通过集成带通滤波器、衰减器和微波放大器的微波前端模块，极大降低了外部线路复杂性，且该集成前端模块体积小，可直接集成到电子学设备中，使得测控脉冲从电子学设备中发生后可直接接入稀释制冷机内，极大简化了外部接线，提升了系统可靠性。</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=02fd591a-9387-4d8e-abef-42688565ec39&amp;shareId=E41F3B0F-9352-71B8-3F94-09F7G7CDE08G&amp;from=EXPORT&amp;signature=1JKZo99fgnMuYC9TeyIO%2BH%2BfMQnWDXkJ55m91pPdA8A%3D&amp;expire=94608000&amp;date=20260529T004228Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=790c2d97-855b-4e0a-9871-d310eb385917&amp;shareId=9822D43G-CCG6-9909-3EB1-2F5994384B2D&amp;from=EXPORT&amp;signature=hpf9T4zP2CQGVclG38u8YABrx6n70ujlX9k7YrglEcI%3D&amp;expire=94608000&amp;date=20260605T003852Z&amp;version=1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
security: remove hardcoded API keys, use DEEPSEEK_API_KEY env var
- config.yaml: key -> env var, unified on DeepSeek API
- config_pro.yaml: switched from Moonshot/Kimi to DeepSeek
- config_en.yaml: switched from Moonshot/Kimi to DeepSeek
- config.py: added _expand_env() for yaml  resolution
- llm_client.py: added _resolve_env() for runtime env var expansion

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/weekly_temp/patents_低温环境系统.xlsx
+++ b/weekly_temp/patents_低温环境系统.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,17 +456,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>一种离子阱及量子计算装置</t>
+          <t>一种超流氦中量子涡旋的精确调控装置及方法</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>华翊博奥(北京)量子科技有限公司</t>
+          <t>浙江大学</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>毛志超 | 蔡明磊 | 梅全鑫 | 赵文定</t>
+          <t>包士然 | 胡应璇 | 黄雯琳 | 骆科旭 | 邱利民</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,34 +476,34 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>本文公开一种离子阱及量子计算装置，包括：一体化基片，制备于一体化基片上的射频电极和直流电极；其中，一体化基片具有轴向的通光开槽。本发明实施例离子阱基于一体化基片设计，消除了温度变化带来的分体错位问题，使得离子阱可以应用于低温环境；通过开放的开槽使离子阱获得了开放式的轴向通光，具有更高的数值孔径，增加了离子阱通光自由度，为实现量子计算的大规模应用提供支持。</t>
+          <t>本发明公开了一种超流氦中量子涡旋的精确调控装置及方法，包括：低温制取与维持系统，包括压缩机、冷水机组、制冷机冷头和液氦室，用于对氦气进行冷却与液化；屏蔽与真空系统，包括真空腔室冷屏、77 K冷屏和4 K冷屏；压力与抽排系统，包括观察室的减压抽空口、减压蝶阀与减压泵组，用于对观察室进行抽排与减压控制；观察与执行单元，包括具有视窗的观察室、布置于观察室内的加热器、由电机驱动的运动格栅、示踪粒子或氦气的注入口以及高速相机；控制系统，与上述各系统电连接并用于协同控制与数据采集。本发明能够在可控低温环境下实现对量子涡旋生成、演化及空间分布进行精确调控与实时观测。</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=812af80b-4741-463b-ab78-d83bde6bb6e8&amp;shareId=52BD9CD7-45FG-8274-0137-9D20G0FC1569&amp;from=EXPORT&amp;signature=5LLF1Ckm3n6GVgymHmMHuQotzmM%2BQT%2Bnh9DyXO%2FReCA%3D&amp;expire=94608000&amp;date=20260710T002807Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=328a8ac1-96bf-45f2-a59b-be5d5e70abb3&amp;shareId=CG922F42-3G7E-9G13-CBD4-870541D3C849&amp;from=EXPORT&amp;signature=GJ%2Fb05PLFk38VfcS%2FCaifEAN0%2BnFnFo1DJSf%2Fw3QdLc%3D&amp;expire=94608000&amp;date=20260717T011040Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>一种兼具耐电晕与导热性能的复合纳米芳纶绝缘纸及其制备与应用</t>
+          <t>超导量子芯片的引线键合方法、制造方法和超导量子芯片</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>四川大学</t>
+          <t>深圳量旋科技有限公司</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>任俊文 | 张稼珵 | 王梓 | 高萌 | 谭淋 | 陈俊雪 | 龙志慧</t>
+          <t>胡金耀</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -513,128 +513,54 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>本发明公开了一种兼具耐电晕与导热性能的复合纳米芳纶绝缘纸及其制备与应用，绝缘纸由芳纶纳米纤维基体以及均匀分散于芳纶纳米纤维基体中的第一功能填料和第二功能填料组成；第一功能填料为经表面功能化处理的氮化硼量子点；第二功能填料为纳米碳化硅；经表面功能化处理的氮化硼量子点的质量为芳纶纳米纤维基体质量的1%~15%，纳米碳化硅质量为芳纶纳米纤维基体质量的0.5%~8%。经表面功能化处理的氮化硼量子点的平均粒径为2nm~10 nm。本发明解决了现有技术缺乏紫外防护机制，填料分布不可控，工艺复杂导热有限的问题，通过电场调控、紫外防护和复合填料优化分布的协同作用，显著提升绝缘纸的耐电晕性能和导热性能。</t>
+          <t>本申请公开了一种超导量子芯片的引线键合方法、制造方法和超导量子芯片。该方法包括：在印刷电路板的第一金属焊盘上方，利用球焊机激发尖端电流融化焊丝形成第一焊球，并与第一金属焊盘熔融共晶形成第一焊点；在超导量子芯片本体的第二金属焊盘上方，同样形成第二焊球并与第二金属焊盘熔融共晶形成第二焊点；利用劈刀从第二焊点处拉出线弧与第一焊点共晶焊接；最后进行退火处理，以消除引线键合引入的残余应力。本申请通过球焊工艺实现超导量子芯片与印刷电路板之间的熔融共晶键合，并结合退火处理消除残余应力，从而提高了焊点在极低温环境下的连接可靠性和超导量子比特的相干性能。</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=3c0b5980-c120-43ac-958a-9b3227662b88&amp;shareId=52BD9CD7-45FG-8274-0137-9D20G0FC1569&amp;from=EXPORT&amp;signature=FycS9fUCKgWV4S3%2Fz0DP0GPwtafHKS%2ByrL9SPMvngXs%3D&amp;expire=94608000&amp;date=20260710T002807Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=4d60c6a1-52d1-445e-a53b-2aee07176021&amp;shareId=CG922F42-3G7E-9G13-CBD4-870541D3C849&amp;from=EXPORT&amp;signature=QzR4N6b2g%2BYZ1a6XW4a7rrg01e12bZfPIVfNsf%2B9KbA%3D&amp;expire=94608000&amp;date=20260717T011040Z&amp;version=1.0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>一种量子点与电磁感应协同配合的电池热管理装置</t>
+          <t>通过部分侧向开启系统轻松进出</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>安徽理工大学</t>
+          <t>液态空气乔治斯克劳帝方法研究开发股份有限公司</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>盛国超 | 朱浩冉 | 张妮 | 冯林涛 | 陈晖</t>
+          <t>GAFFET, LUC | GUIA, OLIVIER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>公开专利</t>
+          <t>授权专利</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>本发明提供一种量子点与电磁感应协同配合的电池热管理装置，涉及电池热管理领域。解决了传统的电池温度调节技术可分为主动和被动两类。被动散热时通过导热材料、相变材料和散热片等使热量传导和存储，虽然结构简单，但控温能力有限。主动散热包括风冷、液冷和制冷剂冷却等。风冷系统散热效率相对较低，适用于电池功率较小的设备的问题，该电池热管理装置是一种双层热管理架构。本发明通过合理设计双层热管理架构，实现了量子点对电池局部温度的精确监控以及利用电磁感应带动磁流体对电池不同区域的差异化冷却，两层系统通过智能控制器协调工作，避免其相互干扰，极大程度的增强了电池热管理在精准温控以及热量调控效果。</t>
+          <t>一种制冷系统,包括:由至少第一壁限定的第一低温腔室,该第一低温腔室与至少一个第一冷源热连接;由至少第二壁限定的第二低温腔室,该第二腔室至少部分地面向所述第一壁,该第二腔室包含于所述第一腔室内并与至少一个第二冷源热连接;其中,所述制冷系统包括至少在第一壁上设置的第一门,该第一门与在第二壁上设置的第二门基本相对,所述第一门和所述第二门的设置方式使得当所述第一门打开时,所述第二门也随之打开。</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=11776872-3db1-45e3-a7ce-1fd48ec7afd6&amp;shareId=52BD9CD7-45FG-8274-0137-9D20G0FC1569&amp;from=EXPORT&amp;signature=3kEVSQrfPlmGj24ygsxuk1XapbqzjpviW7xD2Vi2L6k%3D&amp;expire=94608000&amp;date=20260710T002807Z&amp;version=1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>超导量子位中的光控制的二能级系统的量子位选择性调谐</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>国际商业机器公司</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SANDBERG, MARTIN O. | FALK, ABRAM L. | BALAKRISHNAN, KARTHIK | ORCUTT, JASON S.</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>授权专利</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>提供了用于减轻量子处理器中的缺陷的影响的方法和系统。减轻系统包括具有多个量子位的量子处理器。该系统包括发光源阵列。每个发光源与量子处理器上的量子位对准。该系统包括控制器,该控制器被配置为接收对量子位的选择并且使得来自发光源阵列的发光源向所选择的量子位发射光。光用于混乱量子处理器中的强耦合的两能级系统(TLS)。</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=64917608-271c-47fc-88fd-50abd7014bb1&amp;shareId=52BD9CD7-45FG-8274-0137-9D20G0FC1569&amp;from=EXPORT&amp;signature=zuCRJ1pqzhJMVHxQQf6WnpIUmJzQH1H41vBtZYX6Hxs%3D&amp;expire=94608000&amp;date=20260710T002807Z&amp;version=1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>共集成谐振隧道二极管和高电子迁移率晶体管</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>国际商业机器公司</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CHA, EUNJUNG | ZOTA, BOGDAN CEZAR | MOSELUND, KIRSTEN EMILIE | HNIDA-GUT, KATARZYNA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>授权专利</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>本文提供的一种或多种装置和/或方法涉及一种用于制造具有共集成RTD和HEMT的半导体器件的方法。该半导体器件可以包括沿衬底共集成的RTD和HEMT。一种制造方法可以包括:提供包含多个HEMT晶体管层的异质结构;在垂直堆叠结构上形成模板结构,该模板结构包括开口、空腔和种子结构,所述种子结构包括种子材料和种子表面;以及从所述种子表面在模板结构的空腔内生长多个RTD二极管层,其中RTD和HEMT沿衬底共集成。</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=d79c53bd-df85-4b34-aaf2-b0d0a448a695&amp;shareId=52BD9CD7-45FG-8274-0137-9D20G0FC1569&amp;from=EXPORT&amp;signature=FiI%2BRLrfMqLhU8XiGlxEeiXKZBNWy%2FNqnCD9LeYiKAk%3D&amp;expire=94608000&amp;date=20260710T002807Z&amp;version=1.0</t>
+          <t>https://analytics.zhihuiya.com/patent-view/abst?patentId=0bbf5322-c2fe-4608-afa5-283fe9534f45&amp;shareId=CG922F42-3G7E-9G13-CBD4-870541D3C849&amp;from=EXPORT&amp;signature=QAfMjsanZO%2F%2FA4mRyKKFu%2BgPvSkkOs5LJvk%2F1%2FwbgjU%3D&amp;expire=94608000&amp;date=20260717T011040Z&amp;version=1.0</t>
         </is>
       </c>
     </row>

</xml_diff>